<commit_message>
feat: full admin CRUD user, 9 kelas, dashboard analytics, forum like polymorphic, synthetic seeder
</commit_message>
<xml_diff>
--- a/DATA SISWA SMP ISLAM RAUDLATUL HIKMAH TP.25.26 (1).xlsx
+++ b/DATA SISWA SMP ISLAM RAUDLATUL HIKMAH TP.25.26 (1).xlsx
@@ -1,24 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\TP 25.26\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\LMS-SMP-Raudlatul\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{14E5C851-C77B-4502-9587-EDFA3ACF8B03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27854150-DE03-4882-B7C3-2CAF5034E797}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="4" xr2:uid="{B0DDDD3C-27D3-48F5-BD61-09AE661DFCAC}"/>
+    <workbookView xWindow="384" yWindow="384" windowWidth="17280" windowHeight="9960" xr2:uid="{B0DDDD3C-27D3-48F5-BD61-09AE661DFCAC}"/>
   </bookViews>
   <sheets>
-    <sheet name="Kelas 7" sheetId="1" r:id="rId1"/>
-    <sheet name="Kelas 8.1" sheetId="2" r:id="rId2"/>
-    <sheet name="Kelas 8.2" sheetId="3" r:id="rId3"/>
-    <sheet name="Kelas 8.3" sheetId="4" r:id="rId4"/>
-    <sheet name="Kelas 9.1" sheetId="5" r:id="rId5"/>
-    <sheet name="Kelas 9.2" sheetId="6" r:id="rId6"/>
+    <sheet name="Kelas 7A" sheetId="1" r:id="rId1"/>
+    <sheet name="Kelas 8A" sheetId="2" r:id="rId2"/>
+    <sheet name="Kelas 8B" sheetId="3" r:id="rId3"/>
+    <sheet name="Kelas 8C" sheetId="4" r:id="rId4"/>
+    <sheet name="Kelas 9A" sheetId="5" r:id="rId5"/>
+    <sheet name="Kelas 9B" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="306" uniqueCount="291">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="307" uniqueCount="292">
   <si>
     <t>No</t>
   </si>
@@ -903,6 +903,9 @@
   </si>
   <si>
     <t>Novi Aryanti</t>
+  </si>
+  <si>
+    <t>S</t>
   </si>
 </sst>
 </file>
@@ -1060,15 +1063,6 @@
   </cellStyleXfs>
   <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1152,6 +1146,15 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1484,453 +1487,453 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F415A204-7BD4-4B47-B590-6FE0C810043F}">
   <dimension ref="A3:C44"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="31.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="31.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" s="29" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" s="29" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="C3" s="29" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="2"/>
-      <c r="B4" s="2"/>
-      <c r="C4" s="2"/>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" s="3"/>
-      <c r="B5" s="3"/>
-      <c r="C5" s="3"/>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" s="4"/>
-      <c r="B6" s="4"/>
-      <c r="C6" s="4"/>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" s="5">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" s="30"/>
+      <c r="B4" s="30"/>
+      <c r="C4" s="30"/>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" s="31"/>
+      <c r="B5" s="31"/>
+      <c r="C5" s="31"/>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" s="1"/>
+      <c r="B6" s="1"/>
+      <c r="C6" s="1"/>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" s="2">
         <v>1</v>
       </c>
-      <c r="B7" s="5">
+      <c r="B7" s="2">
         <v>2</v>
       </c>
-      <c r="C7" s="5">
+      <c r="C7" s="2">
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A8" s="6">
+    <row r="8" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A8" s="3">
         <v>1</v>
       </c>
-      <c r="B8" s="7" t="s">
+      <c r="B8" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="C8" s="8" t="s">
+      <c r="C8" s="5" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A9" s="6">
+    <row r="9" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A9" s="3">
         <v>2</v>
       </c>
-      <c r="B9" s="7" t="s">
+      <c r="B9" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="C9" s="8" t="s">
+      <c r="C9" s="5" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A10" s="6">
+    <row r="10" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A10" s="3">
         <v>3</v>
       </c>
-      <c r="B10" s="7" t="s">
+      <c r="B10" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C10" s="8" t="s">
+      <c r="C10" s="5" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A11" s="6">
+    <row r="11" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A11" s="3">
         <v>4</v>
       </c>
-      <c r="B11" s="7" t="s">
+      <c r="B11" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="C11" s="8" t="s">
+      <c r="C11" s="5" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A12" s="6">
+    <row r="12" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A12" s="3">
         <v>5</v>
       </c>
-      <c r="B12" s="7" t="s">
+      <c r="B12" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="C12" s="8" t="s">
+      <c r="C12" s="5" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A13" s="6">
+    <row r="13" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A13" s="3">
         <v>6</v>
       </c>
-      <c r="B13" s="7" t="s">
+      <c r="B13" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="C13" s="8" t="s">
+      <c r="C13" s="5" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A14" s="6">
+    <row r="14" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A14" s="3">
         <v>7</v>
       </c>
-      <c r="B14" s="7" t="s">
+      <c r="B14" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="C14" s="8" t="s">
+      <c r="C14" s="5" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A15" s="6">
+    <row r="15" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A15" s="3">
         <v>8</v>
       </c>
-      <c r="B15" s="7" t="s">
+      <c r="B15" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="C15" s="8" t="s">
+      <c r="C15" s="5" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A16" s="6">
+    <row r="16" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A16" s="3">
         <v>9</v>
       </c>
-      <c r="B16" s="7" t="s">
+      <c r="B16" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="C16" s="8" t="s">
+      <c r="C16" s="5" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A17" s="6">
+    <row r="17" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A17" s="3">
         <v>10</v>
       </c>
-      <c r="B17" s="7" t="s">
+      <c r="B17" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="C17" s="8" t="s">
+      <c r="C17" s="5" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="18" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A18" s="6">
+    <row r="18" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A18" s="3">
         <v>11</v>
       </c>
-      <c r="B18" s="7" t="s">
+      <c r="B18" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="C18" s="8" t="s">
+      <c r="C18" s="5" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="19" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A19" s="6">
+    <row r="19" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A19" s="3">
         <v>12</v>
       </c>
-      <c r="B19" s="7" t="s">
+      <c r="B19" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="C19" s="8" t="s">
+      <c r="C19" s="5" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="20" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A20" s="6">
+    <row r="20" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A20" s="3">
         <v>13</v>
       </c>
-      <c r="B20" s="7" t="s">
+      <c r="B20" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="C20" s="8" t="s">
+      <c r="C20" s="5" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="21" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A21" s="6">
+    <row r="21" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A21" s="3">
         <v>14</v>
       </c>
-      <c r="B21" s="7" t="s">
+      <c r="B21" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="C21" s="8" t="s">
+      <c r="C21" s="5" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="22" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A22" s="6">
+    <row r="22" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A22" s="3">
         <v>15</v>
       </c>
-      <c r="B22" s="7" t="s">
+      <c r="B22" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="C22" s="8" t="s">
+      <c r="C22" s="5" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="23" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A23" s="6">
+    <row r="23" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A23" s="3">
         <v>16</v>
       </c>
-      <c r="B23" s="7" t="s">
+      <c r="B23" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="C23" s="8" t="s">
+      <c r="C23" s="5" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="24" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A24" s="6">
+    <row r="24" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A24" s="3">
         <v>17</v>
       </c>
-      <c r="B24" s="7" t="s">
+      <c r="B24" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="C24" s="8" t="s">
+      <c r="C24" s="5" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="25" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A25" s="6">
+    <row r="25" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A25" s="3">
         <v>18</v>
       </c>
-      <c r="B25" s="7" t="s">
+      <c r="B25" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="C25" s="8" t="s">
+      <c r="C25" s="5" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="26" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A26" s="6">
+    <row r="26" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A26" s="3">
         <v>19</v>
       </c>
-      <c r="B26" s="7" t="s">
+      <c r="B26" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="C26" s="8" t="s">
+      <c r="C26" s="5" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="27" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A27" s="6">
+    <row r="27" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A27" s="3">
         <v>20</v>
       </c>
-      <c r="B27" s="7" t="s">
+      <c r="B27" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="C27" s="8" t="s">
+      <c r="C27" s="5" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="28" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A28" s="6">
+    <row r="28" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A28" s="3">
         <v>21</v>
       </c>
-      <c r="B28" s="7" t="s">
+      <c r="B28" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="C28" s="8" t="s">
+      <c r="C28" s="5" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="29" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A29" s="6">
+    <row r="29" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A29" s="3">
         <v>22</v>
       </c>
-      <c r="B29" s="7" t="s">
+      <c r="B29" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="C29" s="8" t="s">
+      <c r="C29" s="5" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="30" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A30" s="6">
+    <row r="30" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A30" s="3">
         <v>23</v>
       </c>
-      <c r="B30" s="7" t="s">
+      <c r="B30" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="C30" s="8" t="s">
+      <c r="C30" s="5" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="31" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A31" s="6">
+    <row r="31" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A31" s="3">
         <v>24</v>
       </c>
-      <c r="B31" s="7" t="s">
+      <c r="B31" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="C31" s="8" t="s">
+      <c r="C31" s="5" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="32" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A32" s="6">
+    <row r="32" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A32" s="3">
         <v>25</v>
       </c>
-      <c r="B32" s="7" t="s">
+      <c r="B32" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="C32" s="8" t="s">
+      <c r="C32" s="5" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="33" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A33" s="6">
+    <row r="33" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A33" s="3">
         <v>26</v>
       </c>
-      <c r="B33" s="7" t="s">
+      <c r="B33" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="C33" s="8" t="s">
+      <c r="C33" s="5" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="34" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A34" s="6">
+    <row r="34" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A34" s="3">
         <v>27</v>
       </c>
-      <c r="B34" s="7" t="s">
+      <c r="B34" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="C34" s="8" t="s">
+      <c r="C34" s="5" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="35" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A35" s="6">
+    <row r="35" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A35" s="3">
         <v>28</v>
       </c>
-      <c r="B35" s="7" t="s">
+      <c r="B35" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="C35" s="8" t="s">
+      <c r="C35" s="5" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="36" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A36" s="6">
+    <row r="36" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A36" s="3">
         <v>29</v>
       </c>
-      <c r="B36" s="7" t="s">
+      <c r="B36" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="C36" s="8" t="s">
+      <c r="C36" s="5" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="37" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A37" s="6">
+    <row r="37" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A37" s="3">
         <v>30</v>
       </c>
-      <c r="B37" s="7" t="s">
+      <c r="B37" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="C37" s="8" t="s">
+      <c r="C37" s="5" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="38" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A38" s="6">
+    <row r="38" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A38" s="3">
         <v>31</v>
       </c>
-      <c r="B38" s="7" t="s">
+      <c r="B38" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="C38" s="8" t="s">
+      <c r="C38" s="5" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="39" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A39" s="6">
+    <row r="39" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A39" s="3">
         <v>32</v>
       </c>
-      <c r="B39" s="7" t="s">
+      <c r="B39" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="C39" s="8" t="s">
+      <c r="C39" s="5" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="40" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A40" s="6">
+    <row r="40" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A40" s="3">
         <v>33</v>
       </c>
-      <c r="B40" s="7" t="s">
+      <c r="B40" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="C40" s="8" t="s">
+      <c r="C40" s="5" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="41" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A41" s="6">
+    <row r="41" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A41" s="3">
         <v>34</v>
       </c>
-      <c r="B41" s="7" t="s">
+      <c r="B41" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="C41" s="8" t="s">
+      <c r="C41" s="5" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="42" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A42" s="6">
+    <row r="42" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A42" s="3">
         <v>35</v>
       </c>
-      <c r="B42" s="7" t="s">
+      <c r="B42" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="C42" s="9" t="s">
+      <c r="C42" s="6" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="43" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A43" s="6">
+    <row r="43" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A43" s="3">
         <v>36</v>
       </c>
-      <c r="B43" s="7" t="s">
+      <c r="B43" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="C43" s="9" t="s">
+      <c r="C43" s="6" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="44" spans="1:3" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A44" s="6">
+    <row r="44" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A44" s="3">
         <v>37</v>
       </c>
-      <c r="B44" s="10" t="s">
+      <c r="B44" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="C44" s="9" t="s">
+      <c r="C44" s="6" t="s">
         <v>76</v>
       </c>
     </row>
@@ -1947,343 +1950,343 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1D598913-0517-4366-A2B3-F65D5CF99AF3}">
   <dimension ref="A3:C34"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="27.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="27.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
+    <row r="3" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="29" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" s="29" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="C3" s="29" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="2"/>
-      <c r="B4" s="2"/>
-      <c r="C4" s="2"/>
-    </row>
-    <row r="5" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="3"/>
-      <c r="B5" s="3"/>
-      <c r="C5" s="3"/>
-    </row>
-    <row r="6" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="4"/>
-      <c r="B6" s="4"/>
-      <c r="C6" s="4"/>
-    </row>
-    <row r="7" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="5">
+    <row r="4" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="30"/>
+      <c r="B4" s="30"/>
+      <c r="C4" s="30"/>
+    </row>
+    <row r="5" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="31"/>
+      <c r="B5" s="31"/>
+      <c r="C5" s="31"/>
+    </row>
+    <row r="6" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="1"/>
+      <c r="B6" s="1"/>
+      <c r="C6" s="1"/>
+    </row>
+    <row r="7" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="2">
         <v>1</v>
       </c>
-      <c r="B7" s="5">
+      <c r="B7" s="2">
         <v>2</v>
       </c>
-      <c r="C7" s="5">
+      <c r="C7" s="2">
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="6">
+    <row r="8" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="3">
         <v>1</v>
       </c>
-      <c r="B8" s="10" t="s">
+      <c r="B8" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="C8" s="8" t="s">
+      <c r="C8" s="5" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="6">
+    <row r="9" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="3">
         <v>2</v>
       </c>
-      <c r="B9" s="7" t="s">
+      <c r="B9" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="C9" s="8" t="s">
+      <c r="C9" s="5" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="6">
+    <row r="10" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="3">
         <v>3</v>
       </c>
-      <c r="B10" s="10" t="s">
+      <c r="B10" s="7" t="s">
         <v>81</v>
       </c>
-      <c r="C10" s="8" t="s">
+      <c r="C10" s="5" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="6">
+    <row r="11" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="3">
         <v>4</v>
       </c>
-      <c r="B11" s="7" t="s">
+      <c r="B11" s="4" t="s">
         <v>83</v>
       </c>
-      <c r="C11" s="8" t="s">
+      <c r="C11" s="5" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="6">
+    <row r="12" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="3">
         <v>5</v>
       </c>
-      <c r="B12" s="10" t="s">
+      <c r="B12" s="7" t="s">
         <v>85</v>
       </c>
-      <c r="C12" s="8" t="s">
+      <c r="C12" s="5" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="6">
+    <row r="13" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="3">
         <v>6</v>
       </c>
-      <c r="B13" s="10" t="s">
+      <c r="B13" s="7" t="s">
         <v>87</v>
       </c>
-      <c r="C13" s="8" t="s">
+      <c r="C13" s="5" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="6">
+    <row r="14" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="3">
         <v>7</v>
       </c>
-      <c r="B14" s="10" t="s">
+      <c r="B14" s="7" t="s">
         <v>89</v>
       </c>
-      <c r="C14" s="8" t="s">
+      <c r="C14" s="5" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="6">
+    <row r="15" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="3">
         <v>8</v>
       </c>
-      <c r="B15" s="10" t="s">
+      <c r="B15" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="C15" s="8" t="s">
+      <c r="C15" s="5" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="6">
+    <row r="16" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="3">
         <v>9</v>
       </c>
-      <c r="B16" s="10" t="s">
+      <c r="B16" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="C16" s="8" t="s">
+      <c r="C16" s="5" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="6">
+    <row r="17" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="3">
         <v>10</v>
       </c>
-      <c r="B17" s="10" t="s">
+      <c r="B17" s="7" t="s">
         <v>95</v>
       </c>
-      <c r="C17" s="8" t="s">
+      <c r="C17" s="5" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="18" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="6">
+    <row r="18" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="3">
         <v>11</v>
       </c>
-      <c r="B18" s="10" t="s">
+      <c r="B18" s="7" t="s">
         <v>97</v>
       </c>
-      <c r="C18" s="8" t="s">
+      <c r="C18" s="5" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="19" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="6">
+    <row r="19" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="3">
         <v>12</v>
       </c>
-      <c r="B19" s="10" t="s">
+      <c r="B19" s="7" t="s">
         <v>99</v>
       </c>
-      <c r="C19" s="8" t="s">
+      <c r="C19" s="5" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="20" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="6">
+    <row r="20" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="3">
         <v>13</v>
       </c>
-      <c r="B20" s="10" t="s">
+      <c r="B20" s="7" t="s">
         <v>101</v>
       </c>
-      <c r="C20" s="8" t="s">
+      <c r="C20" s="5" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="21" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="6">
+    <row r="21" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="3">
         <v>14</v>
       </c>
-      <c r="B21" s="7" t="s">
+      <c r="B21" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="C21" s="8" t="s">
+      <c r="C21" s="5" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="22" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="6">
+    <row r="22" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="3">
         <v>15</v>
       </c>
-      <c r="B22" s="11" t="s">
+      <c r="B22" s="8" t="s">
         <v>105</v>
       </c>
-      <c r="C22" s="12" t="s">
+      <c r="C22" s="9" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="23" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="6">
+    <row r="23" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="3">
         <v>16</v>
       </c>
-      <c r="B23" s="10" t="s">
+      <c r="B23" s="7" t="s">
         <v>107</v>
       </c>
-      <c r="C23" s="8" t="s">
+      <c r="C23" s="5" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="24" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="6">
+    <row r="24" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="3">
         <v>17</v>
       </c>
-      <c r="B24" s="10" t="s">
+      <c r="B24" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="C24" s="8" t="s">
+      <c r="C24" s="5" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="25" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="6">
+    <row r="25" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="3">
         <v>18</v>
       </c>
-      <c r="B25" s="10" t="s">
+      <c r="B25" s="7" t="s">
         <v>111</v>
       </c>
-      <c r="C25" s="8" t="s">
+      <c r="C25" s="5" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="26" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="6">
+    <row r="26" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="3">
         <v>19</v>
       </c>
-      <c r="B26" s="10" t="s">
+      <c r="B26" s="7" t="s">
         <v>113</v>
       </c>
-      <c r="C26" s="8" t="s">
+      <c r="C26" s="5" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="27" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="6">
+    <row r="27" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="3">
         <v>20</v>
       </c>
-      <c r="B27" s="10" t="s">
+      <c r="B27" s="7" t="s">
         <v>115</v>
       </c>
-      <c r="C27" s="8" t="s">
+      <c r="C27" s="5" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="28" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="6">
+    <row r="28" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="3">
         <v>21</v>
       </c>
-      <c r="B28" s="10" t="s">
+      <c r="B28" s="7" t="s">
         <v>117</v>
       </c>
-      <c r="C28" s="8" t="s">
+      <c r="C28" s="5" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="29" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="6">
+    <row r="29" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="3">
         <v>22</v>
       </c>
-      <c r="B29" s="10" t="s">
+      <c r="B29" s="7" t="s">
         <v>119</v>
       </c>
-      <c r="C29" s="8" t="s">
+      <c r="C29" s="5" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="30" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="6">
+    <row r="30" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="3">
         <v>23</v>
       </c>
-      <c r="B30" s="10" t="s">
+      <c r="B30" s="7" t="s">
         <v>121</v>
       </c>
-      <c r="C30" s="8" t="s">
+      <c r="C30" s="5" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="31" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="6">
+    <row r="31" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A31" s="3">
         <v>24</v>
       </c>
-      <c r="B31" s="10" t="s">
+      <c r="B31" s="7" t="s">
         <v>123</v>
       </c>
-      <c r="C31" s="8" t="s">
+      <c r="C31" s="5" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="32" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="6">
+    <row r="32" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A32" s="3">
         <v>25</v>
       </c>
-      <c r="B32" s="10" t="s">
+      <c r="B32" s="7" t="s">
         <v>125</v>
       </c>
-      <c r="C32" s="8" t="s">
+      <c r="C32" s="5" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="33" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="6">
+    <row r="33" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A33" s="3">
         <v>26</v>
       </c>
-      <c r="B33" s="10" t="s">
+      <c r="B33" s="7" t="s">
         <v>127</v>
       </c>
-      <c r="C33" s="8" t="s">
+      <c r="C33" s="5" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="34" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="6">
+    <row r="34" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A34" s="3">
         <v>27</v>
       </c>
-      <c r="B34" s="10" t="s">
+      <c r="B34" s="7" t="s">
         <v>129</v>
       </c>
-      <c r="C34" s="8" t="s">
+      <c r="C34" s="5" t="s">
         <v>130</v>
       </c>
     </row>
@@ -2300,321 +2303,321 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E50BB95C-9706-47E4-8212-4DC8A7A85EB6}">
   <dimension ref="A3:C32"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="22.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
+    <row r="3" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="29" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" s="29" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="C3" s="29" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="2"/>
-      <c r="B4" s="2"/>
-      <c r="C4" s="2"/>
-    </row>
-    <row r="5" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="3"/>
-      <c r="B5" s="3"/>
-      <c r="C5" s="3"/>
-    </row>
-    <row r="6" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="4"/>
-      <c r="B6" s="4"/>
-      <c r="C6" s="4"/>
-    </row>
-    <row r="7" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="5">
+    <row r="4" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="30"/>
+      <c r="B4" s="30"/>
+      <c r="C4" s="30"/>
+    </row>
+    <row r="5" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="31"/>
+      <c r="B5" s="31"/>
+      <c r="C5" s="31"/>
+    </row>
+    <row r="6" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="1"/>
+      <c r="B6" s="1"/>
+      <c r="C6" s="1"/>
+    </row>
+    <row r="7" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="2">
         <v>1</v>
       </c>
-      <c r="B7" s="5">
+      <c r="B7" s="2">
         <v>2</v>
       </c>
-      <c r="C7" s="5">
+      <c r="C7" s="2">
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="6">
+    <row r="8" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="3">
         <v>1</v>
       </c>
-      <c r="B8" s="10" t="s">
+      <c r="B8" s="7" t="s">
         <v>131</v>
       </c>
-      <c r="C8" s="8" t="s">
+      <c r="C8" s="5" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="6">
+    <row r="9" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="3">
         <v>2</v>
       </c>
-      <c r="B9" s="10" t="s">
+      <c r="B9" s="7" t="s">
         <v>133</v>
       </c>
-      <c r="C9" s="8" t="s">
+      <c r="C9" s="5" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="6">
+    <row r="10" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="3">
         <v>3</v>
       </c>
-      <c r="B10" s="7" t="s">
+      <c r="B10" s="4" t="s">
         <v>135</v>
       </c>
-      <c r="C10" s="8" t="s">
+      <c r="C10" s="5" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="6">
+    <row r="11" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="3">
         <v>4</v>
       </c>
-      <c r="B11" s="10" t="s">
+      <c r="B11" s="7" t="s">
         <v>137</v>
       </c>
-      <c r="C11" s="8" t="s">
+      <c r="C11" s="5" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="6">
+    <row r="12" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="3">
         <v>5</v>
       </c>
-      <c r="B12" s="10" t="s">
+      <c r="B12" s="7" t="s">
         <v>139</v>
       </c>
-      <c r="C12" s="8" t="s">
+      <c r="C12" s="5" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="6">
+    <row r="13" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="3">
         <v>6</v>
       </c>
-      <c r="B13" s="11" t="s">
+      <c r="B13" s="8" t="s">
         <v>141</v>
       </c>
-      <c r="C13" s="12" t="s">
+      <c r="C13" s="9" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="6">
+    <row r="14" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="3">
         <v>7</v>
       </c>
-      <c r="B14" s="10" t="s">
+      <c r="B14" s="7" t="s">
         <v>143</v>
       </c>
-      <c r="C14" s="8" t="s">
+      <c r="C14" s="5" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="6">
+    <row r="15" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="3">
         <v>8</v>
       </c>
-      <c r="B15" s="10" t="s">
+      <c r="B15" s="7" t="s">
         <v>145</v>
       </c>
-      <c r="C15" s="8" t="s">
+      <c r="C15" s="5" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="6">
+    <row r="16" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="3">
         <v>9</v>
       </c>
-      <c r="B16" s="10" t="s">
+      <c r="B16" s="7" t="s">
         <v>147</v>
       </c>
-      <c r="C16" s="8" t="s">
+      <c r="C16" s="5" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="6">
+    <row r="17" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="3">
         <v>10</v>
       </c>
-      <c r="B17" s="11" t="s">
+      <c r="B17" s="8" t="s">
         <v>149</v>
       </c>
-      <c r="C17" s="12" t="s">
+      <c r="C17" s="9" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="18" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="6">
+    <row r="18" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="3">
         <v>11</v>
       </c>
-      <c r="B18" s="10" t="s">
+      <c r="B18" s="7" t="s">
         <v>151</v>
       </c>
-      <c r="C18" s="8" t="s">
+      <c r="C18" s="5" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="19" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="6">
+    <row r="19" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="3">
         <v>12</v>
       </c>
-      <c r="B19" s="11" t="s">
+      <c r="B19" s="8" t="s">
         <v>153</v>
       </c>
-      <c r="C19" s="12" t="s">
+      <c r="C19" s="9" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="20" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="6">
+    <row r="20" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="3">
         <v>13</v>
       </c>
-      <c r="B20" s="10" t="s">
+      <c r="B20" s="7" t="s">
         <v>155</v>
       </c>
-      <c r="C20" s="8" t="s">
+      <c r="C20" s="5" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="21" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="6">
+    <row r="21" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="3">
         <v>14</v>
       </c>
-      <c r="B21" s="10" t="s">
+      <c r="B21" s="7" t="s">
         <v>157</v>
       </c>
-      <c r="C21" s="8" t="s">
+      <c r="C21" s="5" t="s">
         <v>158</v>
       </c>
     </row>
-    <row r="22" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="6">
+    <row r="22" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="3">
         <v>15</v>
       </c>
-      <c r="B22" s="10" t="s">
+      <c r="B22" s="7" t="s">
         <v>159</v>
       </c>
-      <c r="C22" s="8" t="s">
+      <c r="C22" s="5" t="s">
         <v>160</v>
       </c>
     </row>
-    <row r="23" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="6">
+    <row r="23" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="3">
         <v>16</v>
       </c>
-      <c r="B23" s="10" t="s">
+      <c r="B23" s="7" t="s">
         <v>161</v>
       </c>
-      <c r="C23" s="8" t="s">
+      <c r="C23" s="5" t="s">
         <v>162</v>
       </c>
     </row>
-    <row r="24" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="6">
+    <row r="24" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="3">
         <v>17</v>
       </c>
-      <c r="B24" s="7" t="s">
+      <c r="B24" s="4" t="s">
         <v>163</v>
       </c>
-      <c r="C24" s="8" t="s">
+      <c r="C24" s="5" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="25" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="6">
+    <row r="25" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="3">
         <v>18</v>
       </c>
-      <c r="B25" s="10" t="s">
+      <c r="B25" s="7" t="s">
         <v>165</v>
       </c>
-      <c r="C25" s="8" t="s">
+      <c r="C25" s="5" t="s">
         <v>166</v>
       </c>
     </row>
-    <row r="26" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="6">
+    <row r="26" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="3">
         <v>19</v>
       </c>
-      <c r="B26" s="10" t="s">
+      <c r="B26" s="7" t="s">
         <v>167</v>
       </c>
-      <c r="C26" s="8" t="s">
+      <c r="C26" s="5" t="s">
         <v>168</v>
       </c>
     </row>
-    <row r="27" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="6">
+    <row r="27" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="3">
         <v>20</v>
       </c>
-      <c r="B27" s="10" t="s">
+      <c r="B27" s="7" t="s">
         <v>169</v>
       </c>
-      <c r="C27" s="8" t="s">
+      <c r="C27" s="5" t="s">
         <v>170</v>
       </c>
     </row>
-    <row r="28" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="6">
+    <row r="28" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="3">
         <v>21</v>
       </c>
-      <c r="B28" s="10" t="s">
+      <c r="B28" s="7" t="s">
         <v>171</v>
       </c>
-      <c r="C28" s="8" t="s">
+      <c r="C28" s="5" t="s">
         <v>172</v>
       </c>
     </row>
-    <row r="29" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="6">
+    <row r="29" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="3">
         <v>22</v>
       </c>
-      <c r="B29" s="10" t="s">
+      <c r="B29" s="7" t="s">
         <v>173</v>
       </c>
-      <c r="C29" s="8" t="s">
+      <c r="C29" s="5" t="s">
         <v>174</v>
       </c>
     </row>
-    <row r="30" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="6">
+    <row r="30" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="3">
         <v>23</v>
       </c>
-      <c r="B30" s="10" t="s">
+      <c r="B30" s="7" t="s">
         <v>175</v>
       </c>
-      <c r="C30" s="8" t="s">
+      <c r="C30" s="5" t="s">
         <v>176</v>
       </c>
     </row>
-    <row r="31" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="6">
+    <row r="31" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A31" s="3">
         <v>24</v>
       </c>
-      <c r="B31" s="10" t="s">
+      <c r="B31" s="7" t="s">
         <v>177</v>
       </c>
-      <c r="C31" s="8" t="s">
+      <c r="C31" s="5" t="s">
         <v>178</v>
       </c>
     </row>
-    <row r="32" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="6">
+    <row r="32" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A32" s="3">
         <v>25</v>
       </c>
-      <c r="B32" s="13" t="s">
+      <c r="B32" s="10" t="s">
         <v>179</v>
       </c>
-      <c r="C32" s="12" t="s">
+      <c r="C32" s="9" t="s">
         <v>180</v>
       </c>
     </row>
@@ -2631,343 +2634,343 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4A8C74BB-1AF5-4ECD-8A13-6C45AB65D3C7}">
   <dimension ref="A3:C34"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="22.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
+    <row r="3" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="29" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" s="29" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="C3" s="29" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="2"/>
-      <c r="B4" s="2"/>
-      <c r="C4" s="2"/>
-    </row>
-    <row r="5" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="3"/>
-      <c r="B5" s="3"/>
-      <c r="C5" s="3"/>
-    </row>
-    <row r="6" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="4"/>
-      <c r="B6" s="4"/>
-      <c r="C6" s="4"/>
-    </row>
-    <row r="7" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="5">
+    <row r="4" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="30"/>
+      <c r="B4" s="30"/>
+      <c r="C4" s="30"/>
+    </row>
+    <row r="5" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="31"/>
+      <c r="B5" s="31"/>
+      <c r="C5" s="31"/>
+    </row>
+    <row r="6" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="1"/>
+      <c r="B6" s="1"/>
+      <c r="C6" s="1"/>
+    </row>
+    <row r="7" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="2">
         <v>1</v>
       </c>
-      <c r="B7" s="5">
+      <c r="B7" s="2">
         <v>2</v>
       </c>
-      <c r="C7" s="5">
+      <c r="C7" s="2">
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="6">
+    <row r="8" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="3">
         <v>1</v>
       </c>
-      <c r="B8" s="10" t="s">
+      <c r="B8" s="7" t="s">
         <v>181</v>
       </c>
-      <c r="C8" s="8" t="s">
+      <c r="C8" s="5" t="s">
         <v>182</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="6">
+    <row r="9" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="3">
         <v>2</v>
       </c>
-      <c r="B9" s="7" t="s">
+      <c r="B9" s="4" t="s">
         <v>183</v>
       </c>
-      <c r="C9" s="8" t="s">
+      <c r="C9" s="5" t="s">
         <v>184</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="6">
+    <row r="10" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="3">
         <v>3</v>
       </c>
-      <c r="B10" s="10" t="s">
+      <c r="B10" s="7" t="s">
         <v>185</v>
       </c>
-      <c r="C10" s="8" t="s">
+      <c r="C10" s="5" t="s">
         <v>186</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="6">
+    <row r="11" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="3">
         <v>4</v>
       </c>
-      <c r="B11" s="10" t="s">
+      <c r="B11" s="7" t="s">
         <v>187</v>
       </c>
-      <c r="C11" s="8" t="s">
+      <c r="C11" s="5" t="s">
         <v>188</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="6">
+    <row r="12" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="3">
         <v>5</v>
       </c>
-      <c r="B12" s="10" t="s">
+      <c r="B12" s="7" t="s">
         <v>189</v>
       </c>
-      <c r="C12" s="8" t="s">
+      <c r="C12" s="5" t="s">
         <v>190</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="6">
+    <row r="13" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="3">
         <v>6</v>
       </c>
-      <c r="B13" s="10" t="s">
+      <c r="B13" s="7" t="s">
         <v>191</v>
       </c>
-      <c r="C13" s="8" t="s">
+      <c r="C13" s="5" t="s">
         <v>192</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="6">
+    <row r="14" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="3">
         <v>7</v>
       </c>
-      <c r="B14" s="10" t="s">
+      <c r="B14" s="7" t="s">
         <v>193</v>
       </c>
-      <c r="C14" s="8" t="s">
+      <c r="C14" s="5" t="s">
         <v>194</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="6">
+    <row r="15" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="3">
         <v>8</v>
       </c>
-      <c r="B15" s="10" t="s">
+      <c r="B15" s="7" t="s">
         <v>195</v>
       </c>
-      <c r="C15" s="8" t="s">
+      <c r="C15" s="5" t="s">
         <v>196</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="6">
+    <row r="16" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="3">
         <v>9</v>
       </c>
-      <c r="B16" s="10" t="s">
+      <c r="B16" s="7" t="s">
         <v>197</v>
       </c>
-      <c r="C16" s="8" t="s">
+      <c r="C16" s="5" t="s">
         <v>198</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="6">
+    <row r="17" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="3">
         <v>10</v>
       </c>
-      <c r="B17" s="10" t="s">
+      <c r="B17" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="C17" s="8" t="s">
+      <c r="C17" s="5" t="s">
         <v>200</v>
       </c>
     </row>
-    <row r="18" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="6">
+    <row r="18" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="3">
         <v>11</v>
       </c>
-      <c r="B18" s="10" t="s">
+      <c r="B18" s="7" t="s">
         <v>201</v>
       </c>
-      <c r="C18" s="8" t="s">
+      <c r="C18" s="5" t="s">
         <v>202</v>
       </c>
     </row>
-    <row r="19" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="6">
+    <row r="19" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="3">
         <v>12</v>
       </c>
-      <c r="B19" s="10" t="s">
+      <c r="B19" s="7" t="s">
         <v>203</v>
       </c>
-      <c r="C19" s="8" t="s">
+      <c r="C19" s="5" t="s">
         <v>204</v>
       </c>
     </row>
-    <row r="20" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="6">
+    <row r="20" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="3">
         <v>13</v>
       </c>
-      <c r="B20" s="10" t="s">
+      <c r="B20" s="7" t="s">
         <v>205</v>
       </c>
-      <c r="C20" s="8" t="s">
+      <c r="C20" s="5" t="s">
         <v>206</v>
       </c>
     </row>
-    <row r="21" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="6">
+    <row r="21" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="3">
         <v>14</v>
       </c>
-      <c r="B21" s="10" t="s">
+      <c r="B21" s="7" t="s">
         <v>207</v>
       </c>
-      <c r="C21" s="8" t="s">
+      <c r="C21" s="5" t="s">
         <v>208</v>
       </c>
     </row>
-    <row r="22" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="6">
+    <row r="22" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="3">
         <v>15</v>
       </c>
-      <c r="B22" s="13" t="s">
+      <c r="B22" s="10" t="s">
         <v>209</v>
       </c>
-      <c r="C22" s="8" t="s">
+      <c r="C22" s="5" t="s">
         <v>210</v>
       </c>
     </row>
-    <row r="23" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="6">
+    <row r="23" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="3">
         <v>16</v>
       </c>
-      <c r="B23" s="10" t="s">
+      <c r="B23" s="7" t="s">
         <v>211</v>
       </c>
-      <c r="C23" s="8" t="s">
+      <c r="C23" s="5" t="s">
         <v>212</v>
       </c>
     </row>
-    <row r="24" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="6">
+    <row r="24" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="3">
         <v>17</v>
       </c>
-      <c r="B24" s="10" t="s">
+      <c r="B24" s="7" t="s">
         <v>213</v>
       </c>
-      <c r="C24" s="8" t="s">
+      <c r="C24" s="5" t="s">
         <v>214</v>
       </c>
     </row>
-    <row r="25" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="6">
+    <row r="25" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="3">
         <v>18</v>
       </c>
-      <c r="B25" s="10" t="s">
+      <c r="B25" s="7" t="s">
         <v>215</v>
       </c>
-      <c r="C25" s="8" t="s">
+      <c r="C25" s="5" t="s">
         <v>216</v>
       </c>
     </row>
-    <row r="26" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="6">
+    <row r="26" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="3">
         <v>19</v>
       </c>
-      <c r="B26" s="10" t="s">
+      <c r="B26" s="7" t="s">
         <v>217</v>
       </c>
-      <c r="C26" s="8" t="s">
+      <c r="C26" s="5" t="s">
         <v>218</v>
       </c>
     </row>
-    <row r="27" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="6">
+    <row r="27" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="3">
         <v>20</v>
       </c>
-      <c r="B27" s="10" t="s">
+      <c r="B27" s="7" t="s">
         <v>219</v>
       </c>
-      <c r="C27" s="8" t="s">
+      <c r="C27" s="5" t="s">
         <v>220</v>
       </c>
     </row>
-    <row r="28" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="6">
+    <row r="28" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="3">
         <v>21</v>
       </c>
-      <c r="B28" s="10" t="s">
+      <c r="B28" s="7" t="s">
         <v>221</v>
       </c>
-      <c r="C28" s="8" t="s">
+      <c r="C28" s="5" t="s">
         <v>222</v>
       </c>
     </row>
-    <row r="29" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="6">
+    <row r="29" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="3">
         <v>22</v>
       </c>
-      <c r="B29" s="10" t="s">
+      <c r="B29" s="7" t="s">
         <v>223</v>
       </c>
-      <c r="C29" s="8" t="s">
+      <c r="C29" s="5" t="s">
         <v>224</v>
       </c>
     </row>
-    <row r="30" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="6">
+    <row r="30" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="3">
         <v>23</v>
       </c>
-      <c r="B30" s="10" t="s">
+      <c r="B30" s="7" t="s">
         <v>225</v>
       </c>
-      <c r="C30" s="8" t="s">
+      <c r="C30" s="5" t="s">
         <v>226</v>
       </c>
     </row>
-    <row r="31" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="6">
+    <row r="31" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A31" s="3">
         <v>24</v>
       </c>
-      <c r="B31" s="10" t="s">
+      <c r="B31" s="7" t="s">
         <v>227</v>
       </c>
-      <c r="C31" s="8" t="s">
+      <c r="C31" s="5" t="s">
         <v>228</v>
       </c>
     </row>
-    <row r="32" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="6">
+    <row r="32" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A32" s="3">
         <v>25</v>
       </c>
-      <c r="B32" s="10" t="s">
+      <c r="B32" s="7" t="s">
         <v>229</v>
       </c>
-      <c r="C32" s="8" t="s">
+      <c r="C32" s="5" t="s">
         <v>230</v>
       </c>
     </row>
-    <row r="33" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="6">
+    <row r="33" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A33" s="3">
         <v>26</v>
       </c>
-      <c r="B33" s="10" t="s">
+      <c r="B33" s="7" t="s">
         <v>231</v>
       </c>
-      <c r="C33" s="8" t="s">
+      <c r="C33" s="5" t="s">
         <v>232</v>
       </c>
     </row>
-    <row r="34" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="6">
+    <row r="34" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A34" s="3">
         <v>27</v>
       </c>
-      <c r="B34" s="7" t="s">
+      <c r="B34" s="4" t="s">
         <v>233</v>
       </c>
-      <c r="C34" s="8" t="s">
+      <c r="C34" s="5" t="s">
         <v>234</v>
       </c>
     </row>
@@ -2983,333 +2986,336 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{55B2D92F-693E-4A53-BBCC-AC355DE81DB4}">
-  <dimension ref="A3:C33"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A3:H33"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="25.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="25.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
+    <row r="3" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="29" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" s="29" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="C3" s="29" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="2"/>
-      <c r="B4" s="2"/>
-      <c r="C4" s="2"/>
-    </row>
-    <row r="5" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="3"/>
-      <c r="B5" s="3"/>
-      <c r="C5" s="3"/>
-    </row>
-    <row r="6" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="4"/>
-      <c r="B6" s="4"/>
-      <c r="C6" s="4"/>
-    </row>
-    <row r="7" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="5">
+    <row r="4" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="30"/>
+      <c r="B4" s="30"/>
+      <c r="C4" s="30"/>
+    </row>
+    <row r="5" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="31"/>
+      <c r="B5" s="31"/>
+      <c r="C5" s="31"/>
+    </row>
+    <row r="6" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="1"/>
+      <c r="B6" s="1"/>
+      <c r="C6" s="1"/>
+    </row>
+    <row r="7" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="2">
         <v>1</v>
       </c>
-      <c r="B7" s="5">
+      <c r="B7" s="2">
         <v>2</v>
       </c>
-      <c r="C7" s="5">
+      <c r="C7" s="2">
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="6">
+    <row r="8" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="3">
         <v>1</v>
       </c>
-      <c r="B8" s="11" t="s">
+      <c r="B8" s="8" t="s">
         <v>235</v>
       </c>
-      <c r="C8" s="14">
+      <c r="C8" s="11">
         <v>23241028</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="6">
+    <row r="9" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="3">
         <v>2</v>
       </c>
-      <c r="B9" s="11" t="s">
+      <c r="B9" s="8" t="s">
         <v>236</v>
       </c>
-      <c r="C9" s="15">
+      <c r="C9" s="12">
         <v>23241014</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="6">
+    <row r="10" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="3">
         <v>3</v>
       </c>
-      <c r="B10" s="11" t="s">
+      <c r="B10" s="8" t="s">
         <v>237</v>
       </c>
-      <c r="C10" s="16">
+      <c r="C10" s="13">
         <v>23241039</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="6">
+    <row r="11" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="3">
         <v>4</v>
       </c>
-      <c r="B11" s="11" t="s">
+      <c r="B11" s="8" t="s">
         <v>238</v>
       </c>
-      <c r="C11" s="15">
+      <c r="C11" s="12">
         <v>23241008</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="6">
+    <row r="12" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="3">
         <v>5</v>
       </c>
-      <c r="B12" s="7" t="s">
+      <c r="B12" s="4" t="s">
         <v>239</v>
       </c>
-      <c r="C12" s="16">
+      <c r="C12" s="13">
         <v>23241018</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="6">
+    <row r="13" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="3">
         <v>6</v>
       </c>
-      <c r="B13" s="11" t="s">
+      <c r="B13" s="8" t="s">
         <v>240</v>
       </c>
-      <c r="C13" s="17">
+      <c r="C13" s="14">
         <v>23241016</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="6">
+    <row r="14" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="3">
         <v>7</v>
       </c>
-      <c r="B14" s="11" t="s">
+      <c r="B14" s="8" t="s">
         <v>241</v>
       </c>
-      <c r="C14" s="16">
+      <c r="C14" s="13">
         <v>23241024</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="6">
+    <row r="15" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="3">
         <v>8</v>
       </c>
-      <c r="B15" s="11" t="s">
+      <c r="B15" s="8" t="s">
         <v>242</v>
       </c>
-      <c r="C15" s="15">
+      <c r="C15" s="12">
         <v>23241029</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="6">
+    <row r="16" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="3">
         <v>9</v>
       </c>
-      <c r="B16" s="11" t="s">
+      <c r="B16" s="8" t="s">
         <v>243</v>
       </c>
-      <c r="C16" s="15">
+      <c r="C16" s="12">
         <v>23241022</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="6">
+    <row r="17" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="3">
         <v>10</v>
       </c>
-      <c r="B17" s="7" t="s">
+      <c r="B17" s="4" t="s">
         <v>244</v>
       </c>
-      <c r="C17" s="16">
+      <c r="C17" s="13">
         <v>23241020</v>
       </c>
     </row>
-    <row r="18" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="6">
+    <row r="18" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="3">
         <v>11</v>
       </c>
-      <c r="B18" s="11" t="s">
+      <c r="B18" s="8" t="s">
         <v>245</v>
       </c>
-      <c r="C18" s="17">
+      <c r="C18" s="14">
         <v>23241036</v>
       </c>
     </row>
-    <row r="19" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="6">
+    <row r="19" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="3">
         <v>12</v>
       </c>
-      <c r="B19" s="11" t="s">
+      <c r="B19" s="8" t="s">
         <v>246</v>
       </c>
-      <c r="C19" s="16">
+      <c r="C19" s="13">
         <v>23241031</v>
       </c>
     </row>
-    <row r="20" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="6">
+    <row r="20" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="3">
         <v>13</v>
       </c>
-      <c r="B20" s="11" t="s">
+      <c r="B20" s="8" t="s">
         <v>247</v>
       </c>
-      <c r="C20" s="16">
+      <c r="C20" s="13">
         <v>23241026</v>
       </c>
     </row>
-    <row r="21" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="6">
+    <row r="21" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="3">
         <v>14</v>
       </c>
-      <c r="B21" s="11" t="s">
+      <c r="B21" s="8" t="s">
         <v>248</v>
       </c>
-      <c r="C21" s="17">
+      <c r="C21" s="14">
         <v>23241017</v>
       </c>
     </row>
-    <row r="22" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="6">
+    <row r="22" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="3">
         <v>15</v>
       </c>
-      <c r="B22" s="11" t="s">
+      <c r="B22" s="8" t="s">
         <v>249</v>
       </c>
-      <c r="C22" s="16">
+      <c r="C22" s="13">
         <v>23241045</v>
       </c>
     </row>
-    <row r="23" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="6">
+    <row r="23" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="3">
         <v>16</v>
       </c>
-      <c r="B23" s="11" t="s">
+      <c r="B23" s="8" t="s">
         <v>250</v>
       </c>
-      <c r="C23" s="15">
+      <c r="C23" s="12">
         <v>23241012</v>
       </c>
     </row>
-    <row r="24" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="6">
+    <row r="24" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="3">
         <v>17</v>
       </c>
-      <c r="B24" s="7" t="s">
+      <c r="B24" s="4" t="s">
         <v>251</v>
       </c>
-      <c r="C24" s="18" t="s">
+      <c r="C24" s="15" t="s">
         <v>252</v>
       </c>
     </row>
-    <row r="25" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="6">
+    <row r="25" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="3">
         <v>18</v>
       </c>
-      <c r="B25" s="11" t="s">
+      <c r="B25" s="8" t="s">
         <v>253</v>
       </c>
-      <c r="C25" s="15">
+      <c r="C25" s="12">
         <v>23241032</v>
       </c>
     </row>
-    <row r="26" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="6">
+    <row r="26" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="3">
         <v>19</v>
       </c>
-      <c r="B26" s="11" t="s">
+      <c r="B26" s="8" t="s">
         <v>254</v>
       </c>
-      <c r="C26" s="16">
+      <c r="C26" s="13">
         <v>23241035</v>
       </c>
     </row>
-    <row r="27" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="6">
+    <row r="27" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="3">
         <v>20</v>
       </c>
-      <c r="B27" s="7" t="s">
+      <c r="B27" s="4" t="s">
         <v>255</v>
       </c>
-      <c r="C27" s="14">
+      <c r="C27" s="11">
         <v>23241006</v>
       </c>
     </row>
-    <row r="28" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="6">
+    <row r="28" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="3">
         <v>21</v>
       </c>
-      <c r="B28" s="7" t="s">
+      <c r="B28" s="4" t="s">
         <v>256</v>
       </c>
-      <c r="C28" s="19" t="s">
+      <c r="C28" s="16" t="s">
         <v>257</v>
       </c>
     </row>
-    <row r="29" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="6">
+    <row r="29" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="3">
         <v>22</v>
       </c>
-      <c r="B29" s="11" t="s">
+      <c r="B29" s="8" t="s">
         <v>258</v>
       </c>
-      <c r="C29" s="17">
+      <c r="C29" s="14">
         <v>23241040</v>
       </c>
     </row>
-    <row r="30" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="6">
+    <row r="30" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="3">
         <v>23</v>
       </c>
-      <c r="B30" s="11" t="s">
+      <c r="B30" s="8" t="s">
         <v>259</v>
       </c>
-      <c r="C30" s="16">
+      <c r="C30" s="13">
         <v>23241033</v>
       </c>
     </row>
-    <row r="31" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="6">
+    <row r="31" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A31" s="3">
         <v>24</v>
       </c>
-      <c r="B31" s="11" t="s">
+      <c r="B31" s="8" t="s">
         <v>260</v>
       </c>
-      <c r="C31" s="8" t="s">
+      <c r="C31" s="5" t="s">
         <v>261</v>
       </c>
     </row>
-    <row r="32" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="6">
+    <row r="32" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A32" s="3">
         <v>25</v>
       </c>
-      <c r="B32" s="13" t="s">
+      <c r="B32" s="10" t="s">
         <v>262</v>
       </c>
-      <c r="C32" s="17">
+      <c r="C32" s="14">
         <v>23241027</v>
       </c>
-    </row>
-    <row r="33" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="6">
+      <c r="H32" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A33" s="3">
         <v>26</v>
       </c>
-      <c r="B33" s="7" t="s">
+      <c r="B33" s="4" t="s">
         <v>263</v>
       </c>
-      <c r="C33" s="8" t="s">
+      <c r="C33" s="5" t="s">
         <v>264</v>
       </c>
     </row>
@@ -3326,13 +3332,13 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3DA4D538-319D-429B-9168-BA0CBFA6B6E8}">
   <dimension ref="A3:C30"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="28.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.88671875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="32" t="s">
         <v>0</v>
       </c>
@@ -3343,282 +3349,282 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" s="33"/>
       <c r="B4" s="33"/>
       <c r="C4" s="33"/>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" s="34"/>
       <c r="B5" s="34"/>
       <c r="C5" s="34"/>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" s="23"/>
-      <c r="B6" s="23"/>
-      <c r="C6" s="23"/>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" s="21">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" s="20"/>
+      <c r="B6" s="20"/>
+      <c r="C6" s="20"/>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" s="18">
         <v>1</v>
       </c>
-      <c r="B7" s="21">
+      <c r="B7" s="18">
         <v>2</v>
       </c>
-      <c r="C7" s="21">
+      <c r="C7" s="18">
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A8" s="20">
+    <row r="8" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A8" s="17">
         <v>1</v>
       </c>
-      <c r="B8" s="26" t="s">
+      <c r="B8" s="23" t="s">
         <v>265</v>
       </c>
-      <c r="C8" s="29">
+      <c r="C8" s="26">
         <v>23241023</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A9" s="20">
+    <row r="9" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A9" s="17">
         <v>2</v>
       </c>
-      <c r="B9" s="25" t="s">
+      <c r="B9" s="22" t="s">
         <v>266</v>
       </c>
-      <c r="C9" s="28">
+      <c r="C9" s="25">
         <v>23241004</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A10" s="20">
+    <row r="10" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A10" s="17">
         <v>3</v>
       </c>
-      <c r="B10" s="26" t="s">
+      <c r="B10" s="23" t="s">
         <v>267</v>
       </c>
-      <c r="C10" s="29">
+      <c r="C10" s="26">
         <v>23241013</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A11" s="20">
+    <row r="11" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A11" s="17">
         <v>4</v>
       </c>
-      <c r="B11" s="26" t="s">
+      <c r="B11" s="23" t="s">
         <v>268</v>
       </c>
-      <c r="C11" s="29">
+      <c r="C11" s="26">
         <v>23241005</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A12" s="20">
+    <row r="12" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A12" s="17">
         <v>5</v>
       </c>
-      <c r="B12" s="25" t="s">
+      <c r="B12" s="22" t="s">
         <v>269</v>
       </c>
-      <c r="C12" s="28">
+      <c r="C12" s="25">
         <v>23241003</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A13" s="20">
+    <row r="13" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A13" s="17">
         <v>6</v>
       </c>
-      <c r="B13" s="25" t="s">
+      <c r="B13" s="22" t="s">
         <v>270</v>
       </c>
-      <c r="C13" s="28">
+      <c r="C13" s="25">
         <v>23241021</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A14" s="20">
+    <row r="14" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A14" s="17">
         <v>7</v>
       </c>
-      <c r="B14" s="26" t="s">
+      <c r="B14" s="23" t="s">
         <v>271</v>
       </c>
-      <c r="C14" s="29">
+      <c r="C14" s="26">
         <v>23241009</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A15" s="20">
+    <row r="15" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A15" s="17">
         <v>8</v>
       </c>
-      <c r="B15" s="26" t="s">
+      <c r="B15" s="23" t="s">
         <v>272</v>
       </c>
-      <c r="C15" s="29">
+      <c r="C15" s="26">
         <v>23241025</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A16" s="20">
+    <row r="16" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A16" s="17">
         <v>9</v>
       </c>
-      <c r="B16" s="25" t="s">
+      <c r="B16" s="22" t="s">
         <v>273</v>
       </c>
-      <c r="C16" s="28">
+      <c r="C16" s="25">
         <v>23241001</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A17" s="20">
+    <row r="17" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A17" s="17">
         <v>10</v>
       </c>
-      <c r="B17" s="25" t="s">
+      <c r="B17" s="22" t="s">
         <v>274</v>
       </c>
-      <c r="C17" s="22">
+      <c r="C17" s="19">
         <v>23241019</v>
       </c>
     </row>
-    <row r="18" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A18" s="20">
+    <row r="18" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A18" s="17">
         <v>11</v>
       </c>
-      <c r="B18" s="26" t="s">
+      <c r="B18" s="23" t="s">
         <v>275</v>
       </c>
-      <c r="C18" s="27">
+      <c r="C18" s="24">
         <v>23241042</v>
       </c>
     </row>
-    <row r="19" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A19" s="20">
+    <row r="19" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A19" s="17">
         <v>12</v>
       </c>
-      <c r="B19" s="25" t="s">
+      <c r="B19" s="22" t="s">
         <v>276</v>
       </c>
-      <c r="C19" s="24" t="s">
+      <c r="C19" s="21" t="s">
         <v>277</v>
       </c>
     </row>
-    <row r="20" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A20" s="20">
+    <row r="20" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A20" s="17">
         <v>13</v>
       </c>
-      <c r="B20" s="26" t="s">
+      <c r="B20" s="23" t="s">
         <v>278</v>
       </c>
-      <c r="C20" s="27">
+      <c r="C20" s="24">
         <v>23241037</v>
       </c>
     </row>
-    <row r="21" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A21" s="20">
+    <row r="21" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A21" s="17">
         <v>14</v>
       </c>
-      <c r="B21" s="26" t="s">
+      <c r="B21" s="23" t="s">
         <v>279</v>
       </c>
-      <c r="C21" s="27">
+      <c r="C21" s="24">
         <v>23241030</v>
       </c>
     </row>
-    <row r="22" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A22" s="20">
+    <row r="22" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A22" s="17">
         <v>15</v>
       </c>
-      <c r="B22" s="25" t="s">
+      <c r="B22" s="22" t="s">
         <v>280</v>
       </c>
-      <c r="C22" s="28">
+      <c r="C22" s="25">
         <v>23241002</v>
       </c>
     </row>
-    <row r="23" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A23" s="20">
+    <row r="23" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A23" s="17">
         <v>16</v>
       </c>
-      <c r="B23" s="26" t="s">
+      <c r="B23" s="23" t="s">
         <v>281</v>
       </c>
-      <c r="C23" s="27">
+      <c r="C23" s="24">
         <v>23241007</v>
       </c>
     </row>
-    <row r="24" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A24" s="20">
+    <row r="24" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A24" s="17">
         <v>17</v>
       </c>
-      <c r="B24" s="26" t="s">
+      <c r="B24" s="23" t="s">
         <v>282</v>
       </c>
-      <c r="C24" s="29">
+      <c r="C24" s="26">
         <v>23241034</v>
       </c>
     </row>
-    <row r="25" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A25" s="20">
+    <row r="25" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A25" s="17">
         <v>18</v>
       </c>
-      <c r="B25" s="31" t="s">
+      <c r="B25" s="28" t="s">
         <v>283</v>
       </c>
-      <c r="C25" s="28">
+      <c r="C25" s="25">
         <v>23241015</v>
       </c>
     </row>
-    <row r="26" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A26" s="20">
+    <row r="26" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A26" s="17">
         <v>19</v>
       </c>
-      <c r="B26" s="26" t="s">
+      <c r="B26" s="23" t="s">
         <v>284</v>
       </c>
-      <c r="C26" s="24" t="s">
+      <c r="C26" s="21" t="s">
         <v>285</v>
       </c>
     </row>
-    <row r="27" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A27" s="20">
+    <row r="27" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A27" s="17">
         <v>20</v>
       </c>
-      <c r="B27" s="25" t="s">
+      <c r="B27" s="22" t="s">
         <v>286</v>
       </c>
-      <c r="C27" s="30" t="s">
+      <c r="C27" s="27" t="s">
         <v>287</v>
       </c>
     </row>
-    <row r="28" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A28" s="20">
+    <row r="28" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A28" s="17">
         <v>21</v>
       </c>
-      <c r="B28" s="26" t="s">
+      <c r="B28" s="23" t="s">
         <v>288</v>
       </c>
-      <c r="C28" s="29">
+      <c r="C28" s="26">
         <v>23241041</v>
       </c>
     </row>
-    <row r="29" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A29" s="20">
+    <row r="29" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A29" s="17">
         <v>22</v>
       </c>
-      <c r="B29" s="25" t="s">
+      <c r="B29" s="22" t="s">
         <v>289</v>
       </c>
-      <c r="C29" s="28">
+      <c r="C29" s="25">
         <v>23241011</v>
       </c>
     </row>
-    <row r="30" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A30" s="20">
+    <row r="30" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A30" s="17">
         <v>23</v>
       </c>
-      <c r="B30" s="26" t="s">
+      <c r="B30" s="23" t="s">
         <v>290</v>
       </c>
-      <c r="C30" s="28">
+      <c r="C30" s="25">
         <v>23241038</v>
       </c>
     </row>

</xml_diff>